<commit_message>
fix: corrected confusion matrix to evaluate all matched scenarios including EntryPointAuthorization and recognize all inconsistency types (PolicyExposure, UnresolvedDownstream) instead of only chain-based inconsistencies
Expanded confusion matrix computation from downstream-only to all matched scenarios to properly evaluate EntryPointAuthorization against policy-exposure ground truth. Fixed predicted-positive detection to recognize any policy_inconsistencies entry regardless of detail shape, preventing
</commit_message>
<xml_diff>
--- a/train-ticket-aitest/first-inconsistency-injection/output/metrics_train-ticket-aitest_first-inconsistency-injection.xlsx
+++ b/train-ticket-aitest/first-inconsistency-injection/output/metrics_train-ticket-aitest_first-inconsistency-injection.xlsx
@@ -1336,17 +1336,17 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>True Positive Rate (TPR)</t>
+          <t>True Negative Rate</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>False Positive Rate (FPR)</t>
+          <t>False Negative Rate</t>
         </is>
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>False Negative Rate (FNR)</t>
+          <t>False Positive Rate</t>
         </is>
       </c>
       <c r="T23" s="2" t="inlineStr">
@@ -1418,47 +1418,47 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>True Positives: correctly flags inconsistency (TP)</t>
+          <t>Cases that correctly captures inconsistency (TN)</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>False Negatives: misses real inconsistency (FN)</t>
+          <t>Cases that missed inconsistency (FP)</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>TPR = TP/(TP+FN)</t>
+          <t>TNR</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>False Positives: false alarm (FP)</t>
+          <t>Cases that incorrectly captures inconsistencies (FN)</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>True Negatives: correctly reports consistent (TN)</t>
+          <t>Cases that tests consistency (TP)</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>FPR = FP/(FP+TN)</t>
+          <t>FNR</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>False Positives: false alarm (FP)</t>
+          <t>Cases that missed inconsistency (FP)</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>True Negatives: correctly reports consistent (TN)</t>
+          <t>Cases that correctly captures inconsistency (TN)</t>
         </is>
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>FNR = FN/(FN+TP)</t>
+          <t>FPR</t>
         </is>
       </c>
       <c r="T24" s="2" t="inlineStr">
@@ -1504,17 +1504,17 @@
         <v/>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J25">
         <f>IF(I25&gt;0,(H25/I25)*100,0)</f>
         <v/>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -1537,18 +1537,18 @@
         <v>0</v>
       </c>
       <c r="R25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S25">
         <f>IF(Q25+R25&gt;0,Q25/(Q25+R25),0)</f>
         <v/>
       </c>
       <c r="T25">
-        <f>IF(K25+N25&gt;0,K25/(K25+N25),0)</f>
+        <f>IF(O25+L25&gt;0,O25/(O25+L25),0)</f>
         <v/>
       </c>
       <c r="U25">
-        <f>IF(K25+L25&gt;0,K25/(K25+L25),0)</f>
+        <f>IF(O25+N25&gt;0,O25/(O25+N25),0)</f>
         <v/>
       </c>
       <c r="V25">
@@ -1583,17 +1583,17 @@
         <v/>
       </c>
       <c r="H26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J26">
         <f>IF(I26&gt;0,(H26/I26)*100,0)</f>
         <v/>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
@@ -1606,7 +1606,7 @@
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P26">
         <f>IF(N26+O26&gt;0,N26/(N26+O26),0)</f>
@@ -1616,18 +1616,18 @@
         <v>0</v>
       </c>
       <c r="R26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S26">
         <f>IF(Q26+R26&gt;0,Q26/(Q26+R26),0)</f>
         <v/>
       </c>
       <c r="T26">
-        <f>IF(K26+N26&gt;0,K26/(K26+N26),0)</f>
+        <f>IF(O26+L26&gt;0,O26/(O26+L26),0)</f>
         <v/>
       </c>
       <c r="U26">
-        <f>IF(K26+L26&gt;0,K26/(K26+L26),0)</f>
+        <f>IF(O26+N26&gt;0,O26/(O26+N26),0)</f>
         <v/>
       </c>
       <c r="V26">
@@ -1662,10 +1662,10 @@
         <v/>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J27">
         <f>IF(I27&gt;0,(H27/I27)*100,0)</f>
@@ -1675,14 +1675,14 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M27">
         <f>IF(K27+L27&gt;0,K27/(K27+L27),0)</f>
         <v/>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
@@ -1692,7 +1692,7 @@
         <v/>
       </c>
       <c r="Q27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -1702,11 +1702,11 @@
         <v/>
       </c>
       <c r="T27">
-        <f>IF(K27+N27&gt;0,K27/(K27+N27),0)</f>
+        <f>IF(O27+L27&gt;0,O27/(O27+L27),0)</f>
         <v/>
       </c>
       <c r="U27">
-        <f>IF(K27+L27&gt;0,K27/(K27+L27),0)</f>
+        <f>IF(O27+N27&gt;0,O27/(O27+N27),0)</f>
         <v/>
       </c>
       <c r="V27">
@@ -1741,17 +1741,17 @@
         <v/>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J28">
         <f>IF(I28&gt;0,(H28/I28)*100,0)</f>
         <v/>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -1774,18 +1774,18 @@
         <v>0</v>
       </c>
       <c r="R28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S28">
         <f>IF(Q28+R28&gt;0,Q28/(Q28+R28),0)</f>
         <v/>
       </c>
       <c r="T28">
-        <f>IF(K28+N28&gt;0,K28/(K28+N28),0)</f>
+        <f>IF(O28+L28&gt;0,O28/(O28+L28),0)</f>
         <v/>
       </c>
       <c r="U28">
-        <f>IF(K28+L28&gt;0,K28/(K28+L28),0)</f>
+        <f>IF(O28+N28&gt;0,O28/(O28+N28),0)</f>
         <v/>
       </c>
       <c r="V28">
@@ -1820,17 +1820,17 @@
         <v/>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J29">
         <f>IF(I29&gt;0,(H29/I29)*100,0)</f>
         <v/>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P29">
         <f>IF(N29+O29&gt;0,N29/(N29+O29),0)</f>
@@ -1853,18 +1853,18 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S29">
         <f>IF(Q29+R29&gt;0,Q29/(Q29+R29),0)</f>
         <v/>
       </c>
       <c r="T29">
-        <f>IF(K29+N29&gt;0,K29/(K29+N29),0)</f>
+        <f>IF(O29+L29&gt;0,O29/(O29+L29),0)</f>
         <v/>
       </c>
       <c r="U29">
-        <f>IF(K29+L29&gt;0,K29/(K29+L29),0)</f>
+        <f>IF(O29+N29&gt;0,O29/(O29+N29),0)</f>
         <v/>
       </c>
       <c r="V29">
@@ -1899,17 +1899,17 @@
         <v/>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J30">
         <f>IF(I30&gt;0,(H30/I30)*100,0)</f>
         <v/>
       </c>
       <c r="K30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L30" t="n">
         <v>0</v>
@@ -1922,7 +1922,7 @@
         <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P30">
         <f>IF(N30+O30&gt;0,N30/(N30+O30),0)</f>
@@ -1932,18 +1932,18 @@
         <v>0</v>
       </c>
       <c r="R30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S30">
         <f>IF(Q30+R30&gt;0,Q30/(Q30+R30),0)</f>
         <v/>
       </c>
       <c r="T30">
-        <f>IF(K30+N30&gt;0,K30/(K30+N30),0)</f>
+        <f>IF(O30+L30&gt;0,O30/(O30+L30),0)</f>
         <v/>
       </c>
       <c r="U30">
-        <f>IF(K30+L30&gt;0,K30/(K30+L30),0)</f>
+        <f>IF(O30+N30&gt;0,O30/(O30+N30),0)</f>
         <v/>
       </c>
       <c r="V30">
@@ -1978,17 +1978,17 @@
         <v/>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J31">
         <f>IF(I31&gt;0,(H31/I31)*100,0)</f>
         <v/>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
@@ -2011,18 +2011,18 @@
         <v>0</v>
       </c>
       <c r="R31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S31">
         <f>IF(Q31+R31&gt;0,Q31/(Q31+R31),0)</f>
         <v/>
       </c>
       <c r="T31">
-        <f>IF(K31+N31&gt;0,K31/(K31+N31),0)</f>
+        <f>IF(O31+L31&gt;0,O31/(O31+L31),0)</f>
         <v/>
       </c>
       <c r="U31">
-        <f>IF(K31+L31&gt;0,K31/(K31+L31),0)</f>
+        <f>IF(O31+N31&gt;0,O31/(O31+N31),0)</f>
         <v/>
       </c>
       <c r="V31">
@@ -2057,17 +2057,17 @@
         <v/>
       </c>
       <c r="H32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J32">
         <f>IF(I32&gt;0,(H32/I32)*100,0)</f>
         <v/>
       </c>
       <c r="K32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
@@ -2080,7 +2080,7 @@
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P32">
         <f>IF(N32+O32&gt;0,N32/(N32+O32),0)</f>
@@ -2090,18 +2090,18 @@
         <v>0</v>
       </c>
       <c r="R32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S32">
         <f>IF(Q32+R32&gt;0,Q32/(Q32+R32),0)</f>
         <v/>
       </c>
       <c r="T32">
-        <f>IF(K32+N32&gt;0,K32/(K32+N32),0)</f>
+        <f>IF(O32+L32&gt;0,O32/(O32+L32),0)</f>
         <v/>
       </c>
       <c r="U32">
-        <f>IF(K32+L32&gt;0,K32/(K32+L32),0)</f>
+        <f>IF(O32+N32&gt;0,O32/(O32+N32),0)</f>
         <v/>
       </c>
       <c r="V32">
@@ -2136,17 +2136,17 @@
         <v/>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J33">
         <f>IF(I33&gt;0,(H33/I33)*100,0)</f>
         <v/>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
         <v>0</v>
@@ -2159,7 +2159,7 @@
         <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P33">
         <f>IF(N33+O33&gt;0,N33/(N33+O33),0)</f>
@@ -2169,18 +2169,18 @@
         <v>0</v>
       </c>
       <c r="R33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S33">
         <f>IF(Q33+R33&gt;0,Q33/(Q33+R33),0)</f>
         <v/>
       </c>
       <c r="T33">
-        <f>IF(K33+N33&gt;0,K33/(K33+N33),0)</f>
+        <f>IF(O33+L33&gt;0,O33/(O33+L33),0)</f>
         <v/>
       </c>
       <c r="U33">
-        <f>IF(K33+L33&gt;0,K33/(K33+L33),0)</f>
+        <f>IF(O33+N33&gt;0,O33/(O33+N33),0)</f>
         <v/>
       </c>
       <c r="V33">
@@ -2215,17 +2215,17 @@
         <v/>
       </c>
       <c r="H34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J34">
         <f>IF(I34&gt;0,(H34/I34)*100,0)</f>
         <v/>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
@@ -2248,18 +2248,18 @@
         <v>0</v>
       </c>
       <c r="R34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S34">
         <f>IF(Q34+R34&gt;0,Q34/(Q34+R34),0)</f>
         <v/>
       </c>
       <c r="T34">
-        <f>IF(K34+N34&gt;0,K34/(K34+N34),0)</f>
+        <f>IF(O34+L34&gt;0,O34/(O34+L34),0)</f>
         <v/>
       </c>
       <c r="U34">
-        <f>IF(K34+L34&gt;0,K34/(K34+L34),0)</f>
+        <f>IF(O34+N34&gt;0,O34/(O34+N34),0)</f>
         <v/>
       </c>
       <c r="V34">
@@ -2294,17 +2294,17 @@
         <v/>
       </c>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J35">
         <f>IF(I35&gt;0,(H35/I35)*100,0)</f>
         <v/>
       </c>
       <c r="K35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
@@ -2317,7 +2317,7 @@
         <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P35">
         <f>IF(N35+O35&gt;0,N35/(N35+O35),0)</f>
@@ -2327,18 +2327,18 @@
         <v>0</v>
       </c>
       <c r="R35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S35">
         <f>IF(Q35+R35&gt;0,Q35/(Q35+R35),0)</f>
         <v/>
       </c>
       <c r="T35">
-        <f>IF(K35+N35&gt;0,K35/(K35+N35),0)</f>
+        <f>IF(O35+L35&gt;0,O35/(O35+L35),0)</f>
         <v/>
       </c>
       <c r="U35">
-        <f>IF(K35+L35&gt;0,K35/(K35+L35),0)</f>
+        <f>IF(O35+N35&gt;0,O35/(O35+N35),0)</f>
         <v/>
       </c>
       <c r="V35">
@@ -2373,17 +2373,17 @@
         <v/>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J36">
         <f>IF(I36&gt;0,(H36/I36)*100,0)</f>
         <v/>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L36" t="n">
         <v>0</v>
@@ -2396,7 +2396,7 @@
         <v>0</v>
       </c>
       <c r="O36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P36">
         <f>IF(N36+O36&gt;0,N36/(N36+O36),0)</f>
@@ -2406,18 +2406,18 @@
         <v>0</v>
       </c>
       <c r="R36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S36">
         <f>IF(Q36+R36&gt;0,Q36/(Q36+R36),0)</f>
         <v/>
       </c>
       <c r="T36">
-        <f>IF(K36+N36&gt;0,K36/(K36+N36),0)</f>
+        <f>IF(O36+L36&gt;0,O36/(O36+L36),0)</f>
         <v/>
       </c>
       <c r="U36">
-        <f>IF(K36+L36&gt;0,K36/(K36+L36),0)</f>
+        <f>IF(O36+N36&gt;0,O36/(O36+N36),0)</f>
         <v/>
       </c>
       <c r="V36">
@@ -2452,17 +2452,17 @@
         <v/>
       </c>
       <c r="H37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J37">
         <f>IF(I37&gt;0,(H37/I37)*100,0)</f>
         <v/>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
@@ -2485,18 +2485,18 @@
         <v>0</v>
       </c>
       <c r="R37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S37">
         <f>IF(Q37+R37&gt;0,Q37/(Q37+R37),0)</f>
         <v/>
       </c>
       <c r="T37">
-        <f>IF(K37+N37&gt;0,K37/(K37+N37),0)</f>
+        <f>IF(O37+L37&gt;0,O37/(O37+L37),0)</f>
         <v/>
       </c>
       <c r="U37">
-        <f>IF(K37+L37&gt;0,K37/(K37+L37),0)</f>
+        <f>IF(O37+N37&gt;0,O37/(O37+N37),0)</f>
         <v/>
       </c>
       <c r="V37">

</xml_diff>